<commit_message>
feat(tools): v2 auditable workbook, round comparison, Makefile targets; fix text stored as formulas
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: f9fd4a8a-033c-4218-b2f1-2c8da428242c
</commit_message>
<xml_diff>
--- a/referencia/pontuacao-e-calculo.xlsx
+++ b/referencia/pontuacao-e-calculo.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C47"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -694,6 +694,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -719,9 +720,10 @@
           <t>Capability score</t>
         </is>
       </c>
-      <c r="C6" s="5">
-        <f> SUMPRODUCT(níveis × pesos) / SUM(pesos)  — apenas questões respondidas entram</f>
-        <v/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>= SUMPRODUCT(níveis × pesos) / SUM(pesos)  — apenas questões respondidas entram</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -730,9 +732,10 @@
           <t>Pillar score</t>
         </is>
       </c>
-      <c r="C7" s="5">
-        <f> SUMPRODUCT(capability_scores × pesos) / SUM(pesos)  — sobre capabilities do pillar</f>
-        <v/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>= SUMPRODUCT(capability_scores × pesos) / SUM(pesos)  — sobre capabilities do pillar</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -741,11 +744,13 @@
           <t>Overall score</t>
         </is>
       </c>
-      <c r="C8" s="5">
-        <f> SUMPRODUCT(TODAS capabilities × pesos) / SUM(pesos)  — NÃO é média dos 3 pillars</f>
-        <v/>
-      </c>
-    </row>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>= SUMPRODUCT(TODAS capabilities × pesos) / SUM(pesos)  — NÃO é média dos 3 pillars</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -801,6 +806,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -868,6 +874,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -935,6 +942,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -978,6 +986,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -991,9 +1000,10 @@
           <t>gap_size</t>
         </is>
       </c>
-      <c r="C36" s="5">
-        <f> target_level − current_score  (descartado se ≤ 0)</f>
-        <v/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>= target_level − current_score  (descartado se ≤ 0)</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1002,9 +1012,10 @@
           <t>priority_score</t>
         </is>
       </c>
-      <c r="C37" s="5">
-        <f> peso_capability × gap_size</f>
-        <v/>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>= peso_capability × gap_size</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1055,6 +1066,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
@@ -1155,6 +1167,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1317,6 +1330,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
@@ -1339,6 +1353,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
@@ -1361,6 +1376,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
@@ -1414,6 +1430,8 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
@@ -1508,6 +1526,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1696,6 +1715,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -1718,6 +1738,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
@@ -1740,6 +1761,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
@@ -1793,6 +1815,8 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
@@ -1887,6 +1911,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -2075,6 +2100,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -2097,6 +2123,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
@@ -2119,6 +2146,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
@@ -2172,6 +2200,8 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
@@ -2241,7 +2271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2268,6 +2298,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="7" t="inlineStr">
         <is>
@@ -2415,6 +2446,8 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="29" t="inlineStr">
         <is>
@@ -2482,6 +2515,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="31" t="inlineStr">
         <is>
@@ -2501,6 +2535,8 @@
       <c r="H15" s="34" t="n"/>
       <c r="I15" s="35" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="36" t="inlineStr">
         <is>

</xml_diff>